<commit_message>
content: update price list export; add Glitter 3-in-1 Builder Gel images
</commit_message>
<xml_diff>
--- a/price-list-export.xlsx
+++ b/price-list-export.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Leeukopf-Website-Official\gelitup-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172CB0B9-D314-4A3E-9F5D-6DE2142CFC7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFE5B35-C2BE-4464-A82C-16DBAC201BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="price-list-export" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2187" uniqueCount="1085">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2187" uniqueCount="1088">
   <si>
     <t>Item Name</t>
   </si>
@@ -3275,6 +3275,15 @@
   </si>
   <si>
     <t>Neon Cat Eye #NCE07 -HTF</t>
+  </si>
+  <si>
+    <t>Premium Builder Gel Blue 20g -HTF</t>
+  </si>
+  <si>
+    <t>Premium Builder Gel Purple 20g -HTF</t>
+  </si>
+  <si>
+    <t>Premium Builder Gel Mint 20g -HTF</t>
   </si>
 </sst>
 </file>
@@ -9375,7 +9384,7 @@
     </row>
     <row r="531" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A531" s="1" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B531" s="1" t="s">
         <v>531</v>
@@ -13019,10 +13028,10 @@
         <v>1068</v>
       </c>
       <c r="B862" s="1" t="s">
-        <v>1068</v>
+        <v>1085</v>
       </c>
       <c r="C862" s="1">
-        <v>24.45</v>
+        <v>19.95</v>
       </c>
     </row>
     <row r="863" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13030,10 +13039,10 @@
         <v>1069</v>
       </c>
       <c r="B863" s="1" t="s">
-        <v>1069</v>
+        <v>1087</v>
       </c>
       <c r="C863" s="1">
-        <v>24.45</v>
+        <v>19.95</v>
       </c>
     </row>
     <row r="864" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13041,10 +13050,10 @@
         <v>1070</v>
       </c>
       <c r="B864" s="1" t="s">
-        <v>1070</v>
+        <v>1086</v>
       </c>
       <c r="C864" s="1">
-        <v>24.45</v>
+        <v>19.95</v>
       </c>
     </row>
     <row r="865" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -14584,7 +14593,7 @@
         <v>991</v>
       </c>
       <c r="C1004" s="1">
-        <v>6</v>
+        <v>8.968</v>
       </c>
     </row>
     <row r="1005" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -14595,7 +14604,7 @@
         <v>992</v>
       </c>
       <c r="C1005" s="1">
-        <v>6</v>
+        <v>8.968</v>
       </c>
     </row>
     <row r="1006" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -14606,7 +14615,7 @@
         <v>993</v>
       </c>
       <c r="C1006" s="1">
-        <v>6</v>
+        <v>8.968</v>
       </c>
     </row>
     <row r="1007" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Hide discontinued colours, add Nail Clips Pack of 5 pricing, show admin order total
Hide GIUP-163 and GIUP-224 from site/B2B/distributor catalogues via hidden-products.json, add Nail Clips Dual Form Pack of 5 -HTF at EUR 3.50 to the B2B price list, and display the computed order total in the admin order view.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/price-list-export.xlsx
+++ b/price-list-export.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Leeukopf-Website-Official\gelitup-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFE5B35-C2BE-4464-A82C-16DBAC201BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289B573A-6D19-40E7-9860-E6E2FFDCB8DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="price-list-export" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2187" uniqueCount="1088">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2189" uniqueCount="1089">
   <si>
     <t>Item Name</t>
   </si>
@@ -3284,6 +3284,9 @@
   </si>
   <si>
     <t>Premium Builder Gel Mint 20g -HTF</t>
+  </si>
+  <si>
+    <t>Nail Clips Dual Form Single -HTF</t>
   </si>
 </sst>
 </file>
@@ -3545,7 +3548,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C1093"/>
+  <dimension ref="A1:C1094"/>
   <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.33203125" customWidth="1"/>
@@ -14062,7 +14065,7 @@
         <v>943</v>
       </c>
       <c r="B956" s="1" t="s">
-        <v>943</v>
+        <v>1088</v>
       </c>
       <c r="C956" s="1">
         <v>0.75</v>
@@ -14070,32 +14073,32 @@
     </row>
     <row r="957" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A957" s="1" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="B957" s="1" t="s">
-        <v>944</v>
+        <v>1088</v>
       </c>
       <c r="C957" s="1">
-        <v>0.72</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="958" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A958" s="1" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="B958" s="1" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="C958" s="1">
-        <v>1.0960000000000001</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="959" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A959" s="1" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="B959" s="1" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="C959" s="1">
         <v>1.0960000000000001</v>
@@ -14103,32 +14106,32 @@
     </row>
     <row r="960" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A960" s="1" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="B960" s="1" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="C960" s="1">
-        <v>0.72</v>
+        <v>1.0960000000000001</v>
       </c>
     </row>
     <row r="961" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A961" s="1" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B961" s="1" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="C961" s="1">
-        <v>3.8079999999999998</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="962" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A962" s="1" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="B962" s="1" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="C962" s="1">
         <v>3.8079999999999998</v>
@@ -14136,10 +14139,10 @@
     </row>
     <row r="963" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A963" s="1" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B963" s="1" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="C963" s="1">
         <v>3.8079999999999998</v>
@@ -14147,10 +14150,10 @@
     </row>
     <row r="964" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A964" s="1" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B964" s="1" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="C964" s="1">
         <v>3.8079999999999998</v>
@@ -14158,21 +14161,21 @@
     </row>
     <row r="965" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A965" s="1" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="B965" s="1" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="C965" s="1">
-        <v>1.0960000000000001</v>
+        <v>3.8079999999999998</v>
       </c>
     </row>
     <row r="966" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A966" s="1" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B966" s="1" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="C966" s="1">
         <v>1.0960000000000001</v>
@@ -14180,43 +14183,43 @@
     </row>
     <row r="967" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A967" s="1" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="B967" s="1" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="C967" s="1">
-        <v>8.6</v>
+        <v>1.0960000000000001</v>
       </c>
     </row>
     <row r="968" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A968" s="1" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="B968" s="1" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="C968" s="1">
-        <v>18</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="969" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A969" s="1" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="B969" s="1" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="C969" s="1">
-        <v>5.82</v>
+        <v>18</v>
       </c>
     </row>
     <row r="970" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A970" s="1" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="B970" s="1" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="C970" s="1">
         <v>5.82</v>
@@ -14224,32 +14227,32 @@
     </row>
     <row r="971" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A971" s="1" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="B971" s="1" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="C971" s="1">
-        <v>4.96</v>
+        <v>5.82</v>
       </c>
     </row>
     <row r="972" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A972" s="1" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="B972" s="1" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="C972" s="1">
-        <v>4.41</v>
+        <v>4.96</v>
       </c>
     </row>
     <row r="973" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A973" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B973" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="C973" s="1">
         <v>4.41</v>
@@ -14257,32 +14260,32 @@
     </row>
     <row r="974" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A974" s="1" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B974" s="1" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="C974" s="1">
-        <v>11.61</v>
+        <v>4.41</v>
       </c>
     </row>
     <row r="975" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A975" s="1" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="B975" s="1" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="C975" s="1">
-        <v>10.904</v>
+        <v>11.61</v>
       </c>
     </row>
     <row r="976" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A976" s="1" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B976" s="1" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="C976" s="1">
         <v>10.904</v>
@@ -14290,10 +14293,10 @@
     </row>
     <row r="977" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A977" s="1" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B977" s="1" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="C977" s="1">
         <v>10.904</v>
@@ -14301,21 +14304,21 @@
     </row>
     <row r="978" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A978" s="1" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B978" s="1" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="C978" s="1">
-        <v>10.26</v>
+        <v>10.904</v>
       </c>
     </row>
     <row r="979" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A979" s="1" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B979" s="1" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="C979" s="1">
         <v>10.26</v>
@@ -14323,21 +14326,21 @@
     </row>
     <row r="980" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A980" s="1" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B980" s="1" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="C980" s="1">
-        <v>16.064</v>
+        <v>10.26</v>
       </c>
     </row>
     <row r="981" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A981" s="1" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="B981" s="1" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="C981" s="1">
         <v>16.064</v>
@@ -14345,10 +14348,10 @@
     </row>
     <row r="982" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A982" s="1" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B982" s="1" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="C982" s="1">
         <v>16.064</v>
@@ -14356,10 +14359,10 @@
     </row>
     <row r="983" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A983" s="1" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B983" s="1" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="C983" s="1">
         <v>16.064</v>
@@ -14367,21 +14370,21 @@
     </row>
     <row r="984" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A984" s="1" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B984" s="1" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="C984" s="1">
-        <v>10.256</v>
+        <v>16.064</v>
       </c>
     </row>
     <row r="985" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A985" s="1" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="B985" s="1" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="C985" s="1">
         <v>10.256</v>
@@ -14389,10 +14392,10 @@
     </row>
     <row r="986" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A986" s="1" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="B986" s="1" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="C986" s="1">
         <v>10.256</v>
@@ -14400,32 +14403,32 @@
     </row>
     <row r="987" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A987" s="1" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="B987" s="1" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="C987" s="1">
-        <v>6.4</v>
+        <v>10.256</v>
       </c>
     </row>
     <row r="988" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A988" s="1" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B988" s="1" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="C988" s="1">
-        <v>5.2</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="989" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A989" s="1" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B989" s="1" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="C989" s="1">
         <v>5.2</v>
@@ -14433,32 +14436,32 @@
     </row>
     <row r="990" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A990" s="1" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="B990" s="1" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="C990" s="1">
-        <v>5.5279999999999996</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="991" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A991" s="1" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="B991" s="1" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="C991" s="1">
-        <v>6.38</v>
+        <v>5.5279999999999996</v>
       </c>
     </row>
     <row r="992" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A992" s="1" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="B992" s="1" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="C992" s="1">
         <v>6.38</v>
@@ -14466,10 +14469,10 @@
     </row>
     <row r="993" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A993" s="1" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="B993" s="1" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="C993" s="1">
         <v>6.38</v>
@@ -14477,10 +14480,10 @@
     </row>
     <row r="994" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A994" s="1" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B994" s="1" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="C994" s="1">
         <v>6.38</v>
@@ -14488,10 +14491,10 @@
     </row>
     <row r="995" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A995" s="1" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="B995" s="1" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="C995" s="1">
         <v>6.38</v>
@@ -14499,10 +14502,10 @@
     </row>
     <row r="996" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A996" s="1" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B996" s="1" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="C996" s="1">
         <v>6.38</v>
@@ -14510,10 +14513,10 @@
     </row>
     <row r="997" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A997" s="1" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="B997" s="1" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="C997" s="1">
         <v>6.38</v>
@@ -14521,21 +14524,21 @@
     </row>
     <row r="998" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A998" s="1" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="B998" s="1" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="C998" s="1">
-        <v>7.7279999999999998</v>
+        <v>6.38</v>
       </c>
     </row>
     <row r="999" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A999" s="1" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="B999" s="1" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="C999" s="1">
         <v>7.7279999999999998</v>
@@ -14543,21 +14546,21 @@
     </row>
     <row r="1000" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1000" s="1" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B1000" s="1" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="C1000" s="1">
-        <v>8.968</v>
+        <v>7.7279999999999998</v>
       </c>
     </row>
     <row r="1001" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1001" s="1" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B1001" s="1" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="C1001" s="1">
         <v>8.968</v>
@@ -14565,10 +14568,10 @@
     </row>
     <row r="1002" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1002" s="1" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="B1002" s="1" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="C1002" s="1">
         <v>8.968</v>
@@ -14576,10 +14579,10 @@
     </row>
     <row r="1003" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1003" s="1" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B1003" s="1" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="C1003" s="1">
         <v>8.968</v>
@@ -14587,10 +14590,10 @@
     </row>
     <row r="1004" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1004" s="1" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="B1004" s="1" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="C1004" s="1">
         <v>8.968</v>
@@ -14598,10 +14601,10 @@
     </row>
     <row r="1005" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1005" s="1" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B1005" s="1" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="C1005" s="1">
         <v>8.968</v>
@@ -14609,10 +14612,10 @@
     </row>
     <row r="1006" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1006" s="1" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B1006" s="1" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="C1006" s="1">
         <v>8.968</v>
@@ -14620,54 +14623,54 @@
     </row>
     <row r="1007" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1007" s="1" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="B1007" s="1" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C1007" s="1">
-        <v>15.91</v>
+        <v>8.968</v>
       </c>
     </row>
     <row r="1008" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1008" s="1" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="B1008" s="1" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="C1008" s="1">
-        <v>5.74</v>
+        <v>15.91</v>
       </c>
     </row>
     <row r="1009" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1009" s="1" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B1009" s="1" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="C1009" s="1">
-        <v>22.576000000000001</v>
+        <v>5.74</v>
       </c>
     </row>
     <row r="1010" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1010" s="1" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="B1010" s="1" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="C1010" s="1">
-        <v>16.064</v>
+        <v>22.576000000000001</v>
       </c>
     </row>
     <row r="1011" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1011" s="1" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B1011" s="1" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="C1011" s="1">
         <v>16.064</v>
@@ -14675,10 +14678,10 @@
     </row>
     <row r="1012" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1012" s="1" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="B1012" s="1" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="C1012" s="1">
         <v>16.064</v>
@@ -14686,21 +14689,21 @@
     </row>
     <row r="1013" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1013" s="1" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="B1013" s="1" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="C1013" s="1">
-        <v>12.832000000000001</v>
+        <v>16.064</v>
       </c>
     </row>
     <row r="1014" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1014" s="1" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="B1014" s="1" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="C1014" s="1">
         <v>12.832000000000001</v>
@@ -14708,10 +14711,10 @@
     </row>
     <row r="1015" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1015" s="1" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B1015" s="1" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="C1015" s="1">
         <v>12.832000000000001</v>
@@ -14719,21 +14722,21 @@
     </row>
     <row r="1016" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1016" s="1" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B1016" s="1" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="C1016" s="1">
-        <v>13.12</v>
+        <v>12.832000000000001</v>
       </c>
     </row>
     <row r="1017" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1017" s="1" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="B1017" s="1" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="C1017" s="1">
         <v>13.12</v>
@@ -14741,10 +14744,10 @@
     </row>
     <row r="1018" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1018" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="B1018" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="C1018" s="1">
         <v>13.12</v>
@@ -14752,10 +14755,10 @@
     </row>
     <row r="1019" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1019" s="1" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B1019" s="1" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="C1019" s="1">
         <v>13.12</v>
@@ -14763,10 +14766,10 @@
     </row>
     <row r="1020" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1020" s="1" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B1020" s="1" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="C1020" s="1">
         <v>13.12</v>
@@ -14774,10 +14777,10 @@
     </row>
     <row r="1021" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1021" s="1" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B1021" s="1" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="C1021" s="1">
         <v>13.12</v>
@@ -14785,54 +14788,54 @@
     </row>
     <row r="1022" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1022" s="1" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B1022" s="1" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="C1022" s="1">
-        <v>13.79</v>
+        <v>13.12</v>
       </c>
     </row>
     <row r="1023" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1023" s="1" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="B1023" s="1" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="C1023" s="1">
-        <v>19.7</v>
+        <v>13.79</v>
       </c>
     </row>
     <row r="1024" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1024" s="1" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="B1024" s="1" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="C1024" s="1">
-        <v>14.128</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="1025" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1025" s="1" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="B1025" s="1" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="C1025" s="1">
-        <v>5.7359999999999998</v>
+        <v>14.128</v>
       </c>
     </row>
     <row r="1026" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1026" s="1" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="B1026" s="1" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="C1026" s="1">
         <v>5.7359999999999998</v>
@@ -14840,10 +14843,10 @@
     </row>
     <row r="1027" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1027" s="1" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="B1027" s="1" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="C1027" s="1">
         <v>5.7359999999999998</v>
@@ -14851,10 +14854,10 @@
     </row>
     <row r="1028" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1028" s="1" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="B1028" s="1" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="C1028" s="1">
         <v>5.7359999999999998</v>
@@ -14862,65 +14865,65 @@
     </row>
     <row r="1029" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1029" s="1" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="B1029" s="1" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="C1029" s="1">
-        <v>5.0960000000000001</v>
+        <v>5.7359999999999998</v>
       </c>
     </row>
     <row r="1030" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1030" s="1" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="B1030" s="1" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="C1030" s="1">
-        <v>6.3840000000000003</v>
+        <v>5.0960000000000001</v>
       </c>
     </row>
     <row r="1031" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1031" s="1" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="B1031" s="1" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="C1031" s="1">
-        <v>7.6719999999999997</v>
+        <v>6.3840000000000003</v>
       </c>
     </row>
     <row r="1032" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1032" s="1" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="B1032" s="1" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="C1032" s="1">
-        <v>8.9600000000000009</v>
+        <v>7.6719999999999997</v>
       </c>
     </row>
     <row r="1033" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1033" s="1" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="B1033" s="1" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="C1033" s="1">
-        <v>6.1760000000000002</v>
+        <v>8.9600000000000009</v>
       </c>
     </row>
     <row r="1034" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1034" s="1" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="B1034" s="1" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="C1034" s="1">
         <v>6.1760000000000002</v>
@@ -14928,10 +14931,10 @@
     </row>
     <row r="1035" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1035" s="1" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="B1035" s="1" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="C1035" s="1">
         <v>6.1760000000000002</v>
@@ -14939,21 +14942,21 @@
     </row>
     <row r="1036" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1036" s="1" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="B1036" s="1" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="C1036" s="1">
-        <v>7.992</v>
+        <v>6.1760000000000002</v>
       </c>
     </row>
     <row r="1037" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1037" s="1" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="B1037" s="1" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="C1037" s="1">
         <v>7.992</v>
@@ -14961,10 +14964,10 @@
     </row>
     <row r="1038" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1038" s="1" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="B1038" s="1" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="C1038" s="1">
         <v>7.992</v>
@@ -14972,21 +14975,21 @@
     </row>
     <row r="1039" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1039" s="1" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="B1039" s="1" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="C1039" s="1">
-        <v>10</v>
+        <v>7.992</v>
       </c>
     </row>
     <row r="1040" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1040" s="1" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B1040" s="1" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="C1040" s="1">
         <v>10</v>
@@ -14994,10 +14997,10 @@
     </row>
     <row r="1041" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1041" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="B1041" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="C1041" s="1">
         <v>10</v>
@@ -15005,54 +15008,54 @@
     </row>
     <row r="1042" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1042" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="B1042" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="C1042" s="1">
-        <v>167.98</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1043" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1043" s="1" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B1043" s="1" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="C1043" s="1">
-        <v>10.4</v>
+        <v>167.98</v>
       </c>
     </row>
     <row r="1044" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1044" s="1" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="B1044" s="1" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="C1044" s="1">
-        <v>58.24</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="1045" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1045" s="1" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B1045" s="1" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="C1045" s="1">
-        <v>7.41</v>
+        <v>58.24</v>
       </c>
     </row>
     <row r="1046" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1046" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="B1046" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="C1046" s="1">
         <v>7.41</v>
@@ -15060,10 +15063,10 @@
     </row>
     <row r="1047" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1047" s="1" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B1047" s="1" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="C1047" s="1">
         <v>7.41</v>
@@ -15071,10 +15074,10 @@
     </row>
     <row r="1048" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1048" s="1" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="B1048" s="1" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="C1048" s="1">
         <v>7.41</v>
@@ -15082,10 +15085,10 @@
     </row>
     <row r="1049" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1049" s="1" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="B1049" s="1" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="C1049" s="1">
         <v>7.41</v>
@@ -15093,21 +15096,21 @@
     </row>
     <row r="1050" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1050" s="1" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="B1050" s="1" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="C1050" s="1">
-        <v>11.3</v>
+        <v>7.41</v>
       </c>
     </row>
     <row r="1051" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1051" s="1" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="B1051" s="1" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="C1051" s="1">
         <v>11.3</v>
@@ -15115,10 +15118,10 @@
     </row>
     <row r="1052" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1052" s="1" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="B1052" s="1" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="C1052" s="1">
         <v>11.3</v>
@@ -15126,10 +15129,10 @@
     </row>
     <row r="1053" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1053" s="1" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="B1053" s="1" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="C1053" s="1">
         <v>11.3</v>
@@ -15137,21 +15140,21 @@
     </row>
     <row r="1054" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1054" s="1" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="B1054" s="1" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="C1054" s="1">
-        <v>9.4</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="1055" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1055" s="1" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B1055" s="1" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="C1055" s="1">
         <v>9.4</v>
@@ -15159,10 +15162,10 @@
     </row>
     <row r="1056" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1056" s="1" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="B1056" s="1" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="C1056" s="1">
         <v>9.4</v>
@@ -15170,10 +15173,10 @@
     </row>
     <row r="1057" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1057" s="1" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="B1057" s="1" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="C1057" s="1">
         <v>9.4</v>
@@ -15181,10 +15184,10 @@
     </row>
     <row r="1058" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1058" s="1" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="B1058" s="1" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="C1058" s="1">
         <v>9.4</v>
@@ -15192,10 +15195,10 @@
     </row>
     <row r="1059" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1059" s="1" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="B1059" s="1" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="C1059" s="1">
         <v>9.4</v>
@@ -15203,21 +15206,21 @@
     </row>
     <row r="1060" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1060" s="1" t="s">
-        <v>830</v>
+        <v>1046</v>
       </c>
       <c r="B1060" s="1" t="s">
-        <v>830</v>
+        <v>1046</v>
       </c>
       <c r="C1060" s="1">
-        <v>12.84</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="1061" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1061" s="1" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="B1061" s="1" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="C1061" s="1">
         <v>12.84</v>
@@ -15225,10 +15228,10 @@
     </row>
     <row r="1062" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1062" s="1" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="B1062" s="1" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="C1062" s="1">
         <v>12.84</v>
@@ -15236,10 +15239,10 @@
     </row>
     <row r="1063" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1063" s="1" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B1063" s="1" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="C1063" s="1">
         <v>12.84</v>
@@ -15247,10 +15250,10 @@
     </row>
     <row r="1064" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1064" s="1" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B1064" s="1" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="C1064" s="1">
         <v>12.84</v>
@@ -15258,32 +15261,32 @@
     </row>
     <row r="1065" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1065" s="1" t="s">
-        <v>1064</v>
+        <v>829</v>
       </c>
       <c r="B1065" s="1" t="s">
-        <v>1064</v>
+        <v>829</v>
       </c>
       <c r="C1065" s="1">
-        <v>8.25</v>
+        <v>12.84</v>
       </c>
     </row>
     <row r="1066" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1066" s="1" t="s">
-        <v>1047</v>
+        <v>1064</v>
       </c>
       <c r="B1066" s="1" t="s">
-        <v>1047</v>
+        <v>1064</v>
       </c>
       <c r="C1066" s="1">
-        <v>7.41</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="1067" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1067" s="1" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B1067" s="1" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="C1067" s="1">
         <v>7.41</v>
@@ -15291,10 +15294,10 @@
     </row>
     <row r="1068" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1068" s="1" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B1068" s="1" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="C1068" s="1">
         <v>7.41</v>
@@ -15302,10 +15305,10 @@
     </row>
     <row r="1069" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1069" s="1" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B1069" s="1" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="C1069" s="1">
         <v>7.41</v>
@@ -15313,10 +15316,10 @@
     </row>
     <row r="1070" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1070" s="1" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B1070" s="1" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="C1070" s="1">
         <v>7.41</v>
@@ -15324,10 +15327,10 @@
     </row>
     <row r="1071" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1071" s="1" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B1071" s="1" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="C1071" s="1">
         <v>7.41</v>
@@ -15335,10 +15338,10 @@
     </row>
     <row r="1072" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1072" s="1" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="B1072" s="1" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="C1072" s="1">
         <v>7.41</v>
@@ -15346,10 +15349,10 @@
     </row>
     <row r="1073" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1073" s="1" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B1073" s="1" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="C1073" s="1">
         <v>7.41</v>
@@ -15357,10 +15360,10 @@
     </row>
     <row r="1074" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1074" s="1" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B1074" s="1" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="C1074" s="1">
         <v>7.41</v>
@@ -15368,10 +15371,10 @@
     </row>
     <row r="1075" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1075" s="1" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B1075" s="1" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="C1075" s="1">
         <v>7.41</v>
@@ -15379,10 +15382,10 @@
     </row>
     <row r="1076" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1076" s="1" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="B1076" s="1" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="C1076" s="1">
         <v>7.41</v>
@@ -15390,10 +15393,10 @@
     </row>
     <row r="1077" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1077" s="1" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B1077" s="1" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="C1077" s="1">
         <v>7.41</v>
@@ -15401,10 +15404,10 @@
     </row>
     <row r="1078" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1078" s="1" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="B1078" s="1" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="C1078" s="1">
         <v>7.41</v>
@@ -15412,10 +15415,10 @@
     </row>
     <row r="1079" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1079" s="1" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B1079" s="1" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="C1079" s="1">
         <v>7.41</v>
@@ -15423,10 +15426,10 @@
     </row>
     <row r="1080" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1080" s="1" t="s">
-        <v>382</v>
+        <v>1060</v>
       </c>
       <c r="B1080" s="1" t="s">
-        <v>382</v>
+        <v>1060</v>
       </c>
       <c r="C1080" s="1">
         <v>7.41</v>
@@ -15434,10 +15437,10 @@
     </row>
     <row r="1081" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1081" s="1" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B1081" s="1" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C1081" s="1">
         <v>7.41</v>
@@ -15445,10 +15448,10 @@
     </row>
     <row r="1082" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1082" s="1" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B1082" s="1" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C1082" s="1">
         <v>7.41</v>
@@ -15456,10 +15459,10 @@
     </row>
     <row r="1083" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1083" s="1" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="B1083" s="1" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="C1083" s="1">
         <v>7.41</v>
@@ -15467,10 +15470,10 @@
     </row>
     <row r="1084" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1084" s="1" t="s">
-        <v>1061</v>
+        <v>389</v>
       </c>
       <c r="B1084" s="1" t="s">
-        <v>1061</v>
+        <v>389</v>
       </c>
       <c r="C1084" s="1">
         <v>7.41</v>
@@ -15478,10 +15481,10 @@
     </row>
     <row r="1085" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1085" s="1" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="B1085" s="1" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="C1085" s="1">
         <v>7.41</v>
@@ -15489,32 +15492,32 @@
     </row>
     <row r="1086" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1086" s="1" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B1086" s="1" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C1086" s="1">
+        <v>7.41</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1087" s="1" t="s">
         <v>1063</v>
       </c>
-      <c r="B1086" s="1" t="s">
+      <c r="B1087" s="1" t="s">
         <v>1063</v>
       </c>
-      <c r="C1086" s="1">
-        <v>7.41</v>
-      </c>
-    </row>
-    <row r="1087" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1087" t="s">
-        <v>1078</v>
-      </c>
-      <c r="B1087" t="s">
-        <v>1078</v>
-      </c>
       <c r="C1087" s="1">
-        <v>13.65</v>
+        <v>7.41</v>
       </c>
     </row>
     <row r="1088" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1088" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="B1088" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="C1088" s="1">
         <v>13.65</v>
@@ -15522,10 +15525,10 @@
     </row>
     <row r="1089" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1089" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="B1089" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="C1089" s="1">
         <v>13.65</v>
@@ -15533,10 +15536,10 @@
     </row>
     <row r="1090" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1090" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="B1090" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="C1090" s="1">
         <v>13.65</v>
@@ -15544,10 +15547,10 @@
     </row>
     <row r="1091" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1091" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="B1091" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="C1091" s="1">
         <v>13.65</v>
@@ -15555,10 +15558,10 @@
     </row>
     <row r="1092" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1092" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B1092" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="C1092" s="1">
         <v>13.65</v>
@@ -15566,12 +15569,23 @@
     </row>
     <row r="1093" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1093" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B1093" t="s">
+        <v>1083</v>
+      </c>
+      <c r="C1093" s="1">
+        <v>13.65</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1094" t="s">
         <v>1084</v>
       </c>
-      <c r="B1093" t="s">
+      <c r="B1094" t="s">
         <v>1084</v>
       </c>
-      <c r="C1093" s="1">
+      <c r="C1094" s="1">
         <v>13.65</v>
       </c>
     </row>

</xml_diff>